<commit_message>
Rett Kenneth-kupongen til delt skoreformat
Resultata låg samanslått ("1-0") i midtkolonnen; Bjarte vil ha heimemål i
D, "-" i midten (E) og bortemål i F. Splitta alle 72 rader. Verdiane er
uendra – berre rett kolonne. App-dataen var alt korrekt.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM Tipping 2026 - Kenneth.xlsx
+++ b/VM Tipping 2026 - Kenneth.xlsx
@@ -776,13 +776,17 @@
           <t>Mexico – Sør-Afrika</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n"/>
+      <c r="D3" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -805,13 +809,17 @@
           <t>Sør-Korea – Tsjekkia</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n"/>
+      <c r="D4" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -834,13 +842,17 @@
           <t>Canada – Bosnia-Hercegovina</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n"/>
+      <c r="D5" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -863,13 +875,17 @@
           <t>USA – Paraguay</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n"/>
+      <c r="D6" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -892,13 +908,17 @@
           <t>Qatar – Sveits</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
+      <c r="D7" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>0-2</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -921,13 +941,17 @@
           <t>Brasil – Marokko</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n"/>
+      <c r="D8" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>4-1</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -950,13 +974,17 @@
           <t>Haiti – Skottland</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n"/>
+      <c r="D9" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>3</v>
+      </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -979,13 +1007,17 @@
           <t>Australia – Tyrkia</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1008,13 +1040,17 @@
           <t>Tyskland – Curaçao</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n"/>
+      <c r="D11" s="7" t="n">
+        <v>5</v>
+      </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>5-0</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1037,13 +1073,17 @@
           <t>Nederland – Japan</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n"/>
+      <c r="D12" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1066,13 +1106,17 @@
           <t>Elfenbenskysten – Ecuador</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n"/>
+      <c r="D13" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1095,13 +1139,17 @@
           <t>Sverige – Tunisia</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n"/>
+      <c r="D14" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1124,13 +1172,17 @@
           <t>Spania – Kapp Verde</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n"/>
+      <c r="D15" s="7" t="n">
+        <v>6</v>
+      </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>6-0</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1153,13 +1205,17 @@
           <t>Belgia – Egypt</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n"/>
+      <c r="D16" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1182,13 +1238,17 @@
           <t>Saudi Arabia – Uruguay</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n"/>
+      <c r="D17" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1211,13 +1271,17 @@
           <t>Iran – New Zealand</t>
         </is>
       </c>
-      <c r="D18" s="9" t="n"/>
+      <c r="D18" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1240,13 +1304,17 @@
           <t>Frankrike – Senegal</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n"/>
+      <c r="D19" s="7" t="n">
+        <v>3</v>
+      </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1269,13 +1337,17 @@
           <t>Irak – Norge</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n"/>
+      <c r="D20" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1298,13 +1370,17 @@
           <t>Argentina – Algerie</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n"/>
+      <c r="D21" s="7" t="n">
+        <v>3</v>
+      </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1327,13 +1403,17 @@
           <t>Østerrike – Jordan</t>
         </is>
       </c>
-      <c r="D22" s="9" t="n"/>
+      <c r="D22" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1356,13 +1436,17 @@
           <t>Portugal – DR Kongo</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n"/>
+      <c r="D23" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1385,13 +1469,17 @@
           <t>England – Kroatia</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n"/>
+      <c r="D24" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>2-2</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1414,13 +1502,17 @@
           <t>Ghana – Panama</t>
         </is>
       </c>
-      <c r="D25" s="9" t="n"/>
+      <c r="D25" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1443,13 +1535,17 @@
           <t>Usbekistan – Colombia</t>
         </is>
       </c>
-      <c r="D26" s="11" t="n"/>
+      <c r="D26" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>0-3</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1472,13 +1568,17 @@
           <t>Tsjekkia – Sør-Afrika</t>
         </is>
       </c>
-      <c r="D27" s="11" t="n"/>
+      <c r="D27" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1501,13 +1601,17 @@
           <t>Sveits – Bosnia-Hercegovina</t>
         </is>
       </c>
-      <c r="D28" s="11" t="n"/>
+      <c r="D28" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1530,13 +1634,17 @@
           <t>Canada – Qatar</t>
         </is>
       </c>
-      <c r="D29" s="11" t="n"/>
+      <c r="D29" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1559,13 +1667,17 @@
           <t>Mexico – Sør-Korea</t>
         </is>
       </c>
-      <c r="D30" s="11" t="n"/>
+      <c r="D30" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F30" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G30" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1588,13 +1700,17 @@
           <t>USA – Australia</t>
         </is>
       </c>
-      <c r="D31" s="11" t="n"/>
+      <c r="D31" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G31" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1617,13 +1733,17 @@
           <t>Skottland – Marokko</t>
         </is>
       </c>
-      <c r="D32" s="11" t="n"/>
+      <c r="D32" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G32" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1646,13 +1766,17 @@
           <t>Brasil – Haiti</t>
         </is>
       </c>
-      <c r="D33" s="11" t="n"/>
+      <c r="D33" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="G33" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1675,13 +1799,17 @@
           <t>Tyrkia – Paraguay</t>
         </is>
       </c>
-      <c r="D34" s="11" t="n"/>
+      <c r="D34" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F34" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G34" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1704,13 +1832,17 @@
           <t>Nederland – Sverige</t>
         </is>
       </c>
-      <c r="D35" s="11" t="n"/>
+      <c r="D35" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1733,13 +1865,17 @@
           <t>Tyskland – Elfenbenskysten</t>
         </is>
       </c>
-      <c r="D36" s="11" t="n"/>
+      <c r="D36" s="11" t="n">
+        <v>3</v>
+      </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="F36" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1762,13 +1898,17 @@
           <t>Ecuador – Curaçao</t>
         </is>
       </c>
-      <c r="D37" s="11" t="n"/>
+      <c r="D37" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="F37" s="11" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="n">
+        <v>0</v>
+      </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1791,13 +1931,17 @@
           <t>Tunisia – Japan</t>
         </is>
       </c>
-      <c r="D38" s="7" t="n"/>
+      <c r="D38" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="G38" s="26" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1820,13 +1964,17 @@
           <t>Spania – Saudi Arabia</t>
         </is>
       </c>
-      <c r="D39" s="9" t="n"/>
+      <c r="D39" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>4-1</t>
-        </is>
-      </c>
-      <c r="F39" s="15" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="G39" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1849,13 +1997,17 @@
           <t>Belgia – Iran</t>
         </is>
       </c>
-      <c r="D40" s="7" t="n"/>
+      <c r="D40" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="G40" s="27" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1878,13 +2030,17 @@
           <t>Uruguay – Kapp Verde</t>
         </is>
       </c>
-      <c r="D41" s="9" t="n"/>
+      <c r="D41" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1907,13 +2063,17 @@
           <t>New Zealand – Egypt</t>
         </is>
       </c>
-      <c r="D42" s="9" t="n"/>
+      <c r="D42" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G42" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1936,13 +2096,17 @@
           <t>Argentina – Østerrike</t>
         </is>
       </c>
-      <c r="D43" s="9" t="n"/>
+      <c r="D43" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G43" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -1965,13 +2129,17 @@
           <t>Frankrike – Irak</t>
         </is>
       </c>
-      <c r="D44" s="9" t="n"/>
+      <c r="D44" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G44" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -1994,13 +2162,17 @@
           <t xml:space="preserve">Norge – Senegal </t>
         </is>
       </c>
-      <c r="D45" s="9" t="n"/>
+      <c r="D45" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G45" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2023,13 +2195,17 @@
           <t>Jordan – Algerie</t>
         </is>
       </c>
-      <c r="D46" s="7" t="n"/>
+      <c r="D46" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="F46" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="G46" s="27" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2052,13 +2228,17 @@
           <t>Portugal – Usbekistan</t>
         </is>
       </c>
-      <c r="D47" s="9" t="n"/>
+      <c r="D47" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G47" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2081,13 +2261,17 @@
           <t>England – Ghana</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n"/>
+      <c r="D48" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F48" s="7" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="G48" s="27" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2110,13 +2294,17 @@
           <t>Panama – Kroatia</t>
         </is>
       </c>
-      <c r="D49" s="9" t="n"/>
+      <c r="D49" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G49" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2139,13 +2327,17 @@
           <t xml:space="preserve">Colombia – DR Kongo </t>
         </is>
       </c>
-      <c r="D50" s="9" t="n"/>
+      <c r="D50" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G50" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2167,13 +2359,17 @@
           <t>Sveits – Canada</t>
         </is>
       </c>
-      <c r="D51" s="9" t="n"/>
+      <c r="D51" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G51" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2195,13 +2391,17 @@
           <t>Bosnia-Hercegovina – Qatar</t>
         </is>
       </c>
-      <c r="D52" s="9" t="n"/>
+      <c r="D52" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G52" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2223,13 +2423,17 @@
           <t>Skottland – Brasil</t>
         </is>
       </c>
-      <c r="D53" s="9" t="n"/>
+      <c r="D53" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="G53" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2251,13 +2455,17 @@
           <t>Marokko – Haiti</t>
         </is>
       </c>
-      <c r="D54" s="9" t="n"/>
+      <c r="D54" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E54" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="F54" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="G54" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2279,13 +2487,17 @@
           <t>Mexico – Tsjekkia</t>
         </is>
       </c>
-      <c r="D55" s="9" t="n"/>
+      <c r="D55" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G55" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2307,13 +2519,17 @@
           <t>Sør-Afrika – Sør-Korea</t>
         </is>
       </c>
-      <c r="D56" s="9" t="n"/>
+      <c r="D56" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E56" s="10" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F56" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G56" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2335,13 +2551,17 @@
           <t>Curaçao – Elfenbenskysten</t>
         </is>
       </c>
-      <c r="D57" s="9" t="n"/>
+      <c r="D57" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
-        </is>
-      </c>
-      <c r="F57" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G57" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2363,13 +2583,17 @@
           <t>Ecuador – Tyskland</t>
         </is>
       </c>
-      <c r="D58" s="9" t="n"/>
+      <c r="D58" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="E58" s="10" t="inlineStr">
         <is>
-          <t>0-3</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="G58" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2391,13 +2615,17 @@
           <t>Tunisia – Nederland</t>
         </is>
       </c>
-      <c r="D59" s="9" t="n"/>
+      <c r="D59" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="F59" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="G59" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2419,13 +2647,17 @@
           <t>Japan – Sverige</t>
         </is>
       </c>
-      <c r="D60" s="9" t="n"/>
+      <c r="D60" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G60" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2447,13 +2679,17 @@
           <t>Tyrkia – USA</t>
         </is>
       </c>
-      <c r="D61" s="9" t="n"/>
+      <c r="D61" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G61" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2475,13 +2711,17 @@
           <t>Paraguay – Australia</t>
         </is>
       </c>
-      <c r="D62" s="9" t="n"/>
+      <c r="D62" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G62" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2503,13 +2743,17 @@
           <t>Norge – Frankrike</t>
         </is>
       </c>
-      <c r="D63" s="9" t="n"/>
+      <c r="D63" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="E63" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G63" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2531,13 +2775,17 @@
           <t>Senegal – Irak</t>
         </is>
       </c>
-      <c r="D64" s="9" t="n"/>
+      <c r="D64" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E64" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F64" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G64" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2559,13 +2807,17 @@
           <t>Kapp Verde – Saudi Arabia</t>
         </is>
       </c>
-      <c r="D65" s="9" t="n"/>
+      <c r="D65" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="E65" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
-        </is>
-      </c>
-      <c r="F65" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G65" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2587,13 +2839,17 @@
           <t>Uruguay – Spania</t>
         </is>
       </c>
-      <c r="D66" s="9" t="n"/>
+      <c r="D66" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="F66" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="G66" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2615,13 +2871,17 @@
           <t>Egypt – Iran</t>
         </is>
       </c>
-      <c r="D67" s="9" t="n"/>
+      <c r="D67" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="E67" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="F67" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G67" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2643,13 +2903,17 @@
           <t>New Zealand – Belgia</t>
         </is>
       </c>
-      <c r="D68" s="9" t="n"/>
+      <c r="D68" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E68" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G68" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2671,13 +2935,17 @@
           <t>Panama – England</t>
         </is>
       </c>
-      <c r="D69" s="9" t="n"/>
+      <c r="D69" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="E69" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G69" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2699,13 +2967,17 @@
           <t>Kroatia – Ghana</t>
         </is>
       </c>
-      <c r="D70" s="9" t="n"/>
+      <c r="D70" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G70" s="17" t="inlineStr">
         <is>
           <t>TV2</t>
@@ -2727,13 +2999,17 @@
           <t>Colombia – Portugal</t>
         </is>
       </c>
-      <c r="D71" s="9" t="n"/>
+      <c r="D71" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E71" s="10" t="inlineStr">
         <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F71" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="G71" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2755,13 +3031,17 @@
           <t>DR Kongo – Usbekistan</t>
         </is>
       </c>
-      <c r="D72" s="9" t="n"/>
+      <c r="D72" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E72" s="10" t="inlineStr">
         <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F72" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G72" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2783,13 +3063,17 @@
           <t>Algerie – Østerrike</t>
         </is>
       </c>
-      <c r="D73" s="9" t="n"/>
+      <c r="D73" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E73" s="10" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F73" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G73" s="17" t="inlineStr">
         <is>
           <t>NRK</t>
@@ -2811,13 +3095,17 @@
           <t>Jordan – Argentina</t>
         </is>
       </c>
-      <c r="D74" s="9" t="n"/>
+      <c r="D74" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="E74" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="n"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="G74" s="17" t="inlineStr">
         <is>
           <t>NRK</t>

</xml_diff>